<commit_message>
added new automation code
</commit_message>
<xml_diff>
--- a/Batch15_Playwright_TypeScript_AI_Curriculum.xlsx
+++ b/Batch15_Playwright_TypeScript_AI_Curriculum.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Trainings\GTM_Playwright_Batch15_24June26\GTM_PlaywrightTS_BATCH15\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1664013F-806D-4DCA-A48E-EC1BA29DFC95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCEC0660-2079-46C3-9BB4-35FD8B4D921A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="122">
   <si>
     <t>Week</t>
   </si>
@@ -344,61 +344,49 @@
     <t>https://demo.invoiceninja.com/</t>
   </si>
   <si>
-    <t>Anish</t>
-  </si>
-  <si>
-    <t>ShreeLatha</t>
-  </si>
-  <si>
-    <t>Neha</t>
-  </si>
-  <si>
-    <t>Surya</t>
-  </si>
-  <si>
-    <t>Soumedra</t>
-  </si>
-  <si>
-    <t>Chetan</t>
-  </si>
-  <si>
-    <t>Tejashvini</t>
-  </si>
-  <si>
-    <t>Pradeep</t>
-  </si>
-  <si>
-    <t>Prateek</t>
-  </si>
-  <si>
-    <t>Mayuri</t>
-  </si>
-  <si>
-    <t>Ankita</t>
-  </si>
-  <si>
-    <t>Amar</t>
-  </si>
-  <si>
-    <t>Pavan</t>
-  </si>
-  <si>
     <t>Akshay</t>
   </si>
   <si>
-    <t>Naveen</t>
-  </si>
-  <si>
-    <t>Chalsa</t>
-  </si>
-  <si>
-    <t>Yuvashree</t>
-  </si>
-  <si>
     <t>https://sqatools.in/playwright-page-object-model/</t>
   </si>
   <si>
     <t>Done</t>
+  </si>
+  <si>
+    <t>Shukrant</t>
+  </si>
+  <si>
+    <t>Nayana</t>
+  </si>
+  <si>
+    <t>Amiet</t>
+  </si>
+  <si>
+    <t>Deepak</t>
+  </si>
+  <si>
+    <t>Kalyani</t>
+  </si>
+  <si>
+    <t>Dhanyashwar</t>
+  </si>
+  <si>
+    <t>Kshitija</t>
+  </si>
+  <si>
+    <t>Shubhangi</t>
+  </si>
+  <si>
+    <t>Jyothi</t>
+  </si>
+  <si>
+    <t>Ashvini</t>
+  </si>
+  <si>
+    <t>Vishwa Shetty</t>
+  </si>
+  <si>
+    <t>Harshal</t>
   </si>
 </sst>
 </file>
@@ -799,7 +787,8 @@
   <cols>
     <col min="1" max="1" width="35" customWidth="1"/>
     <col min="2" max="2" width="15.44140625" customWidth="1"/>
-    <col min="3" max="4" width="35" customWidth="1"/>
+    <col min="3" max="3" width="35" customWidth="1"/>
+    <col min="4" max="4" width="22.77734375" customWidth="1"/>
     <col min="6" max="6" width="37.44140625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -837,7 +826,7 @@
         <v>6</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
@@ -852,7 +841,7 @@
         <v>6</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
@@ -867,7 +856,7 @@
         <v>6</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
@@ -882,7 +871,7 @@
         <v>6</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
@@ -897,7 +886,7 @@
         <v>6</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
@@ -914,7 +903,7 @@
         <v>6</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
@@ -929,7 +918,7 @@
         <v>6</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
@@ -944,7 +933,7 @@
         <v>6</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
@@ -959,7 +948,7 @@
         <v>6</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
@@ -974,7 +963,7 @@
         <v>6</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
@@ -991,7 +980,7 @@
         <v>6</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
@@ -1006,7 +995,7 @@
         <v>6</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
@@ -1021,7 +1010,7 @@
         <v>6</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
@@ -1036,7 +1025,7 @@
         <v>6</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
@@ -1051,7 +1040,7 @@
         <v>6</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -1068,7 +1057,7 @@
         <v>6</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
@@ -1083,7 +1072,7 @@
         <v>6</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -1098,7 +1087,7 @@
         <v>6</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
@@ -1126,7 +1115,7 @@
         <v>6</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
@@ -1143,7 +1132,7 @@
         <v>6</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
@@ -1158,7 +1147,7 @@
         <v>6</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
@@ -1173,7 +1162,7 @@
         <v>6</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
@@ -1188,7 +1177,7 @@
         <v>6</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
@@ -1203,7 +1192,7 @@
         <v>6</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
@@ -1220,7 +1209,7 @@
         <v>6</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
@@ -1234,7 +1223,9 @@
       <c r="D28" t="s">
         <v>6</v>
       </c>
-      <c r="E28" s="3"/>
+      <c r="E28" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="8"/>
@@ -1247,7 +1238,9 @@
       <c r="D29" t="s">
         <v>6</v>
       </c>
-      <c r="E29" s="3"/>
+      <c r="E29" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="8"/>
@@ -1257,14 +1250,18 @@
       <c r="D30" t="s">
         <v>6</v>
       </c>
-      <c r="E30" s="3"/>
+      <c r="E30" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="8"/>
       <c r="C31" t="s">
         <v>88</v>
       </c>
-      <c r="E31" s="3"/>
+      <c r="E31" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="8"/>
@@ -1278,7 +1275,7 @@
         <v>6</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
@@ -1292,7 +1289,9 @@
       <c r="D33" t="s">
         <v>6</v>
       </c>
-      <c r="E33" s="3"/>
+      <c r="E33" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
@@ -1307,7 +1306,9 @@
       <c r="D34" t="s">
         <v>6</v>
       </c>
-      <c r="E34" s="3"/>
+      <c r="E34" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="8"/>
@@ -1320,7 +1321,9 @@
       <c r="D35" t="s">
         <v>6</v>
       </c>
-      <c r="E35" s="3"/>
+      <c r="E35" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="8"/>
@@ -1333,7 +1336,9 @@
       <c r="D36" t="s">
         <v>6</v>
       </c>
-      <c r="E36" s="3"/>
+      <c r="E36" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="8"/>
@@ -1346,7 +1351,9 @@
       <c r="D37" t="s">
         <v>6</v>
       </c>
-      <c r="E37" s="3"/>
+      <c r="E37" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="8"/>
@@ -1359,7 +1366,9 @@
       <c r="D38" t="s">
         <v>6</v>
       </c>
-      <c r="E38" s="3"/>
+      <c r="E38" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="8" t="s">
@@ -1374,7 +1383,9 @@
       <c r="D39" t="s">
         <v>6</v>
       </c>
-      <c r="E39" s="3"/>
+      <c r="E39" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="8"/>
@@ -1387,7 +1398,9 @@
       <c r="D40" t="s">
         <v>6</v>
       </c>
-      <c r="E40" s="3"/>
+      <c r="E40" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="8"/>
@@ -1400,7 +1413,9 @@
       <c r="D41" t="s">
         <v>6</v>
       </c>
-      <c r="E41" s="3"/>
+      <c r="E41" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="8"/>
@@ -1413,7 +1428,9 @@
       <c r="D42" t="s">
         <v>6</v>
       </c>
-      <c r="E42" s="3"/>
+      <c r="E42" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="8"/>
@@ -1426,7 +1443,9 @@
       <c r="D43" t="s">
         <v>6</v>
       </c>
-      <c r="E43" s="3"/>
+      <c r="E43" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="8" t="s">
@@ -1441,7 +1460,9 @@
       <c r="D44" t="s">
         <v>6</v>
       </c>
-      <c r="E44" s="3"/>
+      <c r="E44" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="8"/>
@@ -1454,7 +1475,9 @@
       <c r="D45" t="s">
         <v>6</v>
       </c>
-      <c r="E45" s="3"/>
+      <c r="E45" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="8"/>
@@ -1467,7 +1490,9 @@
       <c r="D46" t="s">
         <v>6</v>
       </c>
-      <c r="E46" s="3"/>
+      <c r="E46" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="8"/>
@@ -1480,7 +1505,9 @@
       <c r="D47" t="s">
         <v>6</v>
       </c>
-      <c r="E47" s="3"/>
+      <c r="E47" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="8"/>
@@ -1493,7 +1520,9 @@
       <c r="D48" t="s">
         <v>6</v>
       </c>
-      <c r="E48" s="3"/>
+      <c r="E48" s="3" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="8" t="s">
@@ -1509,7 +1538,7 @@
         <v>6</v>
       </c>
       <c r="E49" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
@@ -1524,7 +1553,7 @@
         <v>6</v>
       </c>
       <c r="E50" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
@@ -1539,7 +1568,7 @@
         <v>6</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
@@ -1554,7 +1583,7 @@
         <v>6</v>
       </c>
       <c r="E52" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
@@ -1569,7 +1598,7 @@
         <v>6</v>
       </c>
       <c r="E53" s="3" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
@@ -1770,8 +1799,8 @@
   <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="53.33203125" customWidth="1"/>
+    <col min="3" max="3" width="58.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
@@ -1793,7 +1822,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C2" t="s">
         <v>95</v>
@@ -1804,7 +1833,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C3" t="s">
         <v>96</v>
@@ -1815,7 +1844,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C4" t="s">
         <v>97</v>
@@ -1826,7 +1855,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C5" t="s">
         <v>95</v>
@@ -1837,7 +1866,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="C6" t="s">
         <v>99</v>
@@ -1848,7 +1877,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C7" t="s">
         <v>100</v>
@@ -1859,7 +1888,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>101</v>
@@ -1870,7 +1899,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C9" t="s">
         <v>102</v>
@@ -1881,7 +1910,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C10" t="s">
         <v>103</v>
@@ -1892,7 +1921,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>116</v>
+        <v>107</v>
       </c>
       <c r="C11" t="s">
         <v>104</v>
@@ -1903,7 +1932,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C12" t="s">
         <v>105</v>
@@ -1914,7 +1943,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C13" t="s">
         <v>106</v>
@@ -1925,7 +1954,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C14" t="s">
         <v>97</v>
@@ -1935,9 +1964,6 @@
       <c r="A15" s="5">
         <v>14</v>
       </c>
-      <c r="B15" t="s">
-        <v>120</v>
-      </c>
       <c r="C15" t="s">
         <v>98</v>
       </c>
@@ -1946,9 +1972,6 @@
       <c r="A16" s="5">
         <v>15</v>
       </c>
-      <c r="B16" t="s">
-        <v>121</v>
-      </c>
       <c r="C16" t="s">
         <v>99</v>
       </c>
@@ -1957,9 +1980,6 @@
       <c r="A17" s="5">
         <v>16</v>
       </c>
-      <c r="B17" t="s">
-        <v>122</v>
-      </c>
       <c r="C17" t="s">
         <v>100</v>
       </c>
@@ -1968,9 +1988,6 @@
       <c r="A18" s="5">
         <v>17</v>
       </c>
-      <c r="B18" t="s">
-        <v>123</v>
-      </c>
       <c r="C18" s="2" t="s">
         <v>101</v>
       </c>
@@ -1981,7 +1998,7 @@
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="5"/>
       <c r="B20" s="7" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">

</xml_diff>